<commit_message>
Remove answer controls from Q10078 materials
</commit_message>
<xml_diff>
--- a/artifacts/任务规格转化.xlsx
+++ b/artifacts/任务规格转化.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="R42dedc07059a43ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="R920a678d2f564aae"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -418,7 +418,7 @@
         <x:v>详情与键盘</x:v>
       </x:c>
       <x:c r="B14" s="5" t="str">
-        <x:v>滚动后打开C1027并读取transcript_count；连续Tab到达五个规定控件，在C1011按Enter打开详情</x:v>
+        <x:v>根据detail_target打开会话并读取transcript_count；使用Tab访问题面规定的控件，按Enter打开获得焦点的会话</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="48" customHeight="1">
@@ -429,12 +429,12 @@
         <x:v>浏览器时区使用Asia/Shanghai，时钟固定为2026-06-18T01:30:00Z，SLA分钟值不读取本机当前时间</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="48" customHeight="1">
+    <x:row r="16" ht="33" customHeight="1">
       <x:c r="A16" s="5" t="str">
         <x:v>截图内容</x:v>
       </x:c>
       <x:c r="B16" s="5" t="str">
-        <x:v>截图取自CASE_AGENT_MINE_BILLING完成S01至S03后，依次显示C1011、C1008、C1030和C1022</x:v>
+        <x:v>截图取自坐席完成指定事件回放后的billing队列，页面会话顺序应与案例报告一致</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="48" customHeight="1">
@@ -442,15 +442,15 @@
         <x:v>完成条件</x:v>
       </x:c>
       <x:c r="B17" s="5" t="str">
-        <x:v>npm run test:e2e返回0，六个目标路径存在，五个case_id均有结果，三份报告能按case_id、event_id和conversation_id互相对照</x:v>
+        <x:v>运行入口生成题面所列报告和截图，三份报告能够按case_id、event_id和conversation_id互相对照</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="48" customHeight="1">
       <x:c r="A18" s="5" t="str">
-        <x:v>可验证点</x:v>
+        <x:v>业务核对点</x:v>
       </x:c>
       <x:c r="B18" s="5" t="str">
-        <x:v>真实Chromium进程、REST路由、WebSocket message、两个角色集合、事件后排序、C1027详情、五步焦点、两条SLA和截图内容</x:v>
+        <x:v>Chromium进程、REST路由、WebSocket message、角色范围、事件后排序、会话详情、键盘焦点、SLA和截图内容</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="48" customHeight="1">

</xml_diff>